<commit_message>
Thêm trạng thái 'Đã cọc' vào tình trạng chuyển khoản
Dropdown giờ có 3 lựa chọn: Đã chuyển khoản (xanh) / Đã cọc (vàng) /
Chưa chuyển khoản (đỏ). Thêm dòng tổng ĐÃ CỌC ở đầu mỗi sheet tháng
và cột ĐÃ CỌC trong bảng tháng, quý, năm của Báo cáo năm.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CPjBCaYmBy58Me5iKx25Jf
</commit_message>
<xml_diff>
--- a/bao-cao-doanh-thu/doanh thu thông tin đơn hàng.xlsx
+++ b/bao-cao-doanh-thu/doanh thu thông tin đơn hàng.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="629" uniqueCount="155">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="638" uniqueCount="158">
   <si>
     <t xml:space="preserve">HƯỚNG DẪN SỬ DỤNG FILE BÁO CÁO DOANH THU - THÔNG TIN ĐƠN HÀNG (THÁNG 6 - THÁNG 12/2026)</t>
   </si>
@@ -66,7 +66,10 @@
     <t xml:space="preserve">   • SỐ LƯỢNG và ĐƠN GIÁ chỉ gõ số (ví dụ 50 và 85000) — không gõ chữ 'cái', 'đ', dấu chấm phẩy.</t>
   </si>
   <si>
-    <t xml:space="preserve">   • TÌNH TRẠNG CHUYỂN KHOẢN: bấm vào ô sẽ có danh sách chọn 'Đã chuyển khoản' / 'Chưa chuyển khoản' (ô tự đổi màu xanh/đỏ).</t>
+    <t xml:space="preserve">   • TÌNH TRẠNG CHUYỂN KHOẢN: bấm vào ô sẽ có danh sách chọn 'Đã chuyển khoản' / 'Đã cọc' / 'Chưa chuyển khoản' (ô tự đổi màu XANH / VÀNG / ĐỎ).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">   • Khách đã cọc: chọn 'Đã cọc' — khi khách thanh toán đủ thì đổi lại thành 'Đã chuyển khoản'. Tổng tiền các đơn đã cọc hiện ở đầu sheet và trong BÁO CÁO NĂM.</t>
   </si>
   <si>
     <t xml:space="preserve">   • Sheet 'Tháng 6' có sẵn 3 dòng VÍ DỤ MẪU (chữ màu xanh dương) — hãy xóa hoặc ghi đè bằng dữ liệu thật của bạn.</t>
@@ -124,6 +127,9 @@
   </si>
   <si>
     <t xml:space="preserve">ĐÃ CHUYỂN KHOẢN (đ):</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ĐÃ CỌC (đ):</t>
   </si>
   <si>
     <t xml:space="preserve">CHƯA CHUYỂN KHOẢN (đ):</t>
@@ -415,6 +421,9 @@
   </si>
   <si>
     <t xml:space="preserve">ĐÃ CK (đ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ĐÃ CỌC (đ)</t>
   </si>
   <si>
     <t xml:space="preserve">CHƯA CK (đ)</t>
@@ -897,11 +906,18 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="3">
     <dxf>
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFEB9C"/>
         </patternFill>
       </fill>
     </dxf>
@@ -950,7 +966,7 @@
       <rgbColor rgb="FF00B0B0"/>
       <rgbColor rgb="FFCCFFFF"/>
       <rgbColor rgb="FFC6EFCE"/>
-      <rgbColor rgb="FFFFFF99"/>
+      <rgbColor rgb="FFFFEB9C"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -1157,7 +1173,7 @@
     <tabColor rgb="FF808080"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:B37"/>
+  <dimension ref="B2:B38"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="3"/>
@@ -1238,15 +1254,15 @@
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B18" s="3"/>
+      <c r="B18" s="3" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B19" s="2" t="s">
-        <v>14</v>
-      </c>
+      <c r="B19" s="3"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B20" s="3" t="s">
+      <c r="B20" s="2" t="s">
         <v>15</v>
       </c>
     </row>
@@ -1256,15 +1272,15 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B22" s="3"/>
+      <c r="B22" s="3" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B23" s="2" t="s">
-        <v>17</v>
-      </c>
+      <c r="B23" s="3"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B24" s="3" t="s">
+      <c r="B24" s="2" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1274,15 +1290,15 @@
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B26" s="3"/>
+      <c r="B26" s="3" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B27" s="2" t="s">
-        <v>20</v>
-      </c>
+      <c r="B27" s="3"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B28" s="3" t="s">
+      <c r="B28" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1297,15 +1313,15 @@
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B31" s="3"/>
+      <c r="B31" s="3" t="s">
+        <v>24</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2" t="s">
-        <v>24</v>
-      </c>
+      <c r="B32" s="3"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B33" s="3" t="s">
+      <c r="B33" s="2" t="s">
         <v>25</v>
       </c>
     </row>
@@ -1315,16 +1331,21 @@
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B35" s="3"/>
+      <c r="B35" s="3" t="s">
+        <v>27</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B36" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="B36" s="3"/>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B37" s="3" t="s">
+      <c r="B37" s="2" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B38" s="3" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1367,7 +1388,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -1385,7 +1406,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -1395,7 +1416,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -1405,31 +1426,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>6000000</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -1457,46 +1486,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46175</v>
@@ -1515,19 +1544,19 @@
         <v>46176</v>
       </c>
       <c r="C10" s="21" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D10" s="21" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="E10" s="22" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="G10" s="21" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="H10" s="23" t="n">
         <v>100</v>
@@ -1540,16 +1569,16 @@
         <v>8500000</v>
       </c>
       <c r="K10" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L10" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M10" s="21" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="N10" s="21" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="P10" s="17" t="n">
         <v>46176</v>
@@ -2364,7 +2393,7 @@
       <c r="M38" s="27"/>
       <c r="N38" s="27"/>
       <c r="P38" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q38" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$37)</f>
@@ -3495,7 +3524,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -3516,46 +3545,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3567,19 +3596,19 @@
         <v>46183</v>
       </c>
       <c r="C92" s="21" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D92" s="21" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E92" s="22" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="F92" s="22" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="G92" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H92" s="23" t="n">
         <v>50</v>
@@ -3592,16 +3621,16 @@
         <v>6000000</v>
       </c>
       <c r="K92" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L92" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M92" s="21" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="N92" s="21" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
     </row>
     <row r="93" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5344,7 +5373,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -5365,46 +5394,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5416,19 +5445,19 @@
         <v>46188</v>
       </c>
       <c r="C174" s="21" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D174" s="21" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E174" s="22" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="F174" s="22" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G174" s="21" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="H174" s="23" t="n">
         <v>200</v>
@@ -5441,16 +5470,16 @@
         <v>7000000</v>
       </c>
       <c r="K174" s="25" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="L174" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M174" s="21" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="N174" s="21" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7193,7 +7222,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -7214,46 +7243,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9017,11 +9046,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -9037,12 +9067,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -9085,7 +9118,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -9103,7 +9136,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -9113,7 +9146,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -9123,31 +9156,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>47000000</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -9175,46 +9216,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46205</v>
@@ -10087,7 +10128,7 @@
       <c r="M39" s="27"/>
       <c r="N39" s="27"/>
       <c r="P39" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q39" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$38)</f>
@@ -11196,7 +11237,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -11217,46 +11258,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13021,7 +13062,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -13042,46 +13083,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13093,19 +13134,19 @@
         <v>46224</v>
       </c>
       <c r="C174" s="21" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D174" s="21" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="E174" s="22" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F174" s="22" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G174" s="21" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="H174" s="23" t="n">
         <v>1000</v>
@@ -13119,11 +13160,11 @@
       </c>
       <c r="K174" s="27"/>
       <c r="L174" s="21" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="M174" s="27"/>
       <c r="N174" s="21" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
     </row>
     <row r="175" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -13135,17 +13176,17 @@
         <v>46224</v>
       </c>
       <c r="C175" s="21" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="D175" s="21" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="E175" s="28"/>
       <c r="F175" s="22" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G175" s="21" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="H175" s="23" t="n">
         <v>1000</v>
@@ -13159,7 +13200,7 @@
       </c>
       <c r="K175" s="27"/>
       <c r="L175" s="21" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M175" s="27"/>
       <c r="N175" s="27"/>
@@ -14882,7 +14923,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -14903,46 +14944,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -16706,11 +16747,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -16726,12 +16768,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -16774,7 +16819,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -16792,7 +16837,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -16802,7 +16847,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -16812,31 +16857,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -16864,46 +16917,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46236</v>
@@ -17776,7 +17829,7 @@
       <c r="M39" s="27"/>
       <c r="N39" s="27"/>
       <c r="P39" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q39" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$38)</f>
@@ -18885,7 +18938,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -18906,46 +18959,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -20710,7 +20763,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -20731,46 +20784,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -22535,7 +22588,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -22556,46 +22609,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -24359,11 +24412,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -24379,12 +24433,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -24427,7 +24484,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -24445,7 +24502,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -24455,7 +24512,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -24465,31 +24522,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -24517,46 +24582,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46267</v>
@@ -25400,7 +25465,7 @@
       <c r="M38" s="27"/>
       <c r="N38" s="27"/>
       <c r="P38" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q38" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$37)</f>
@@ -26531,7 +26596,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -26552,46 +26617,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -28356,7 +28421,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -28377,46 +28442,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -30181,7 +30246,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -30202,46 +30267,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -32005,11 +32070,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -32025,12 +32091,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -32073,7 +32142,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -32091,7 +32160,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -32101,7 +32170,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -32111,31 +32180,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -32163,46 +32240,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46297</v>
@@ -33075,7 +33152,7 @@
       <c r="M39" s="27"/>
       <c r="N39" s="27"/>
       <c r="P39" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q39" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$38)</f>
@@ -34184,7 +34261,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -34205,46 +34282,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -36009,7 +36086,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -36030,46 +36107,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -37834,7 +37911,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -37855,46 +37932,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -39658,11 +39735,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -39678,12 +39756,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -39726,7 +39807,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -39744,7 +39825,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -39754,7 +39835,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -39764,31 +39845,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -39816,46 +39905,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46328</v>
@@ -40699,7 +40788,7 @@
       <c r="M38" s="27"/>
       <c r="N38" s="27"/>
       <c r="P38" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q38" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$37)</f>
@@ -41830,7 +41919,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -41851,46 +41940,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -43655,7 +43744,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -43676,46 +43765,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -45480,7 +45569,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -45501,46 +45590,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -47304,11 +47393,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -47324,12 +47414,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -47372,7 +47465,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -47390,7 +47483,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B3" s="11" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C3" s="11"/>
       <c r="D3" s="12" t="n">
@@ -47400,7 +47493,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B4" s="11" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C4" s="11"/>
       <c r="D4" s="12" t="n">
@@ -47410,31 +47503,39 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B5" s="11" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C5" s="11"/>
       <c r="D5" s="12" t="n">
+        <f aca="false">SUMIF($L$10:$L$335,"Đã cọc",$J$10:$J$335)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B6" s="11" t="s">
+        <v>34</v>
+      </c>
+      <c r="C6" s="11"/>
+      <c r="D6" s="12" t="n">
         <f aca="false">SUMIF($L$10:$L$335,"Chưa chuyển khoản",$J$10:$J$335)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="P6" s="13" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="Q6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P7" s="14" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="Q7" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="15" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B8" s="15"/>
       <c r="C8" s="15"/>
@@ -47462,46 +47563,46 @@
     </row>
     <row r="9" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H9" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I9" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J9" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K9" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L9" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M9" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N9" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="P9" s="17" t="n">
         <v>46358</v>
@@ -48374,7 +48475,7 @@
       <c r="M39" s="27"/>
       <c r="N39" s="27"/>
       <c r="P39" s="31" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="Q39" s="32" t="n">
         <f aca="false">SUM($Q$8:$Q$38)</f>
@@ -49483,7 +49584,7 @@
     </row>
     <row r="90" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A90" s="33" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B90" s="33"/>
       <c r="C90" s="33"/>
@@ -49504,46 +49605,46 @@
     </row>
     <row r="91" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A91" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B91" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C91" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D91" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E91" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F91" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G91" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H91" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I91" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J91" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K91" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L91" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M91" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N91" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="92" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -51308,7 +51409,7 @@
     </row>
     <row r="172" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A172" s="15" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B172" s="15"/>
       <c r="C172" s="15"/>
@@ -51329,46 +51430,46 @@
     </row>
     <row r="173" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A173" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B173" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C173" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D173" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E173" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F173" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G173" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H173" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I173" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J173" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K173" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L173" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M173" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N173" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="174" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -53133,7 +53234,7 @@
     </row>
     <row r="254" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A254" s="33" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B254" s="33"/>
       <c r="C254" s="33"/>
@@ -53154,46 +53255,46 @@
     </row>
     <row r="255" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A255" s="14" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B255" s="14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C255" s="14" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D255" s="14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="E255" s="14" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F255" s="14" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G255" s="14" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="H255" s="14" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="I255" s="14" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="J255" s="14" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="K255" s="14" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="L255" s="14" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="M255" s="14" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="N255" s="14" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="256" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -54957,11 +55058,12 @@
       <c r="N335" s="27"/>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="14">
     <mergeCell ref="A1:N1"/>
     <mergeCell ref="B3:C3"/>
     <mergeCell ref="B4:C4"/>
     <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="P6:Q6"/>
     <mergeCell ref="A8:J8"/>
     <mergeCell ref="K8:N8"/>
@@ -54977,12 +55079,15 @@
       <formula>"Đã chuyển khoản"</formula>
     </cfRule>
     <cfRule type="cellIs" priority="3" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>"Đã cọc"</formula>
+    </cfRule>
+    <cfRule type="cellIs" priority="4" operator="equal" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>"Chưa chuyển khoản"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản hoặc Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
-      <formula1>"Đã chuyển khoản,Chưa chuyển khoản"</formula1>
+    <dataValidation allowBlank="true" error="Chọn: Đã chuyển khoản / Đã cọc / Chưa chuyển khoản" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="L10:L89 L92:L171 L174:L253 L256:L335" type="list">
+      <formula1>"Đã chuyển khoản,Đã cọc,Chưa chuyển khoản"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
@@ -55002,7 +55107,7 @@
     <tabColor rgb="FF1F4E78"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:I36"/>
+  <dimension ref="A1:J36"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="11"/>
@@ -55010,12 +55115,13 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="17"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="7" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="8" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -55028,7 +55134,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="35" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B3" s="35"/>
       <c r="C3" s="35"/>
@@ -55036,7 +55142,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="36" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B4" s="36"/>
       <c r="C4" s="37" t="n">
@@ -55049,60 +55155,64 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="38" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B5" s="38"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="35" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B7" s="35"/>
       <c r="C7" s="35"/>
       <c r="D7" s="35"/>
       <c r="E7" s="35"/>
       <c r="F7" s="35" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G7" s="35"/>
       <c r="H7" s="35"/>
       <c r="I7" s="35"/>
+      <c r="J7" s="35"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B8" s="14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="C8" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="D8" s="14" t="s">
-        <v>127</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="F8" s="14" t="s">
-        <v>124</v>
-      </c>
       <c r="G8" s="14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="I8" s="14" t="s">
-        <v>129</v>
+        <v>131</v>
+      </c>
+      <c r="J8" s="14" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="39" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B9" s="39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C9" s="40" t="n">
         <v>46174</v>
@@ -55115,7 +55225,7 @@
         <v>8500000</v>
       </c>
       <c r="F9" s="42" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="G9" s="43" t="n">
         <f aca="false">'Tháng 6'!$D$3</f>
@@ -55127,15 +55237,19 @@
       </c>
       <c r="I9" s="43" t="n">
         <f aca="false">'Tháng 6'!$D$5</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="43" t="n">
+        <f aca="false">'Tháng 6'!$D$6</f>
         <v>6000000</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="39" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C10" s="40" t="n">
         <v>46181</v>
@@ -55148,7 +55262,7 @@
         <v>6000000</v>
       </c>
       <c r="F10" s="42" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="G10" s="43" t="n">
         <f aca="false">'Tháng 7'!$D$3</f>
@@ -55160,15 +55274,19 @@
       </c>
       <c r="I10" s="43" t="n">
         <f aca="false">'Tháng 7'!$D$5</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="43" t="n">
+        <f aca="false">'Tháng 7'!$D$6</f>
         <v>47000000</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="39" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C11" s="40" t="n">
         <v>46188</v>
@@ -55181,7 +55299,7 @@
         <v>7000000</v>
       </c>
       <c r="F11" s="42" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="G11" s="43" t="n">
         <f aca="false">'Tháng 8'!$D$3</f>
@@ -55195,13 +55313,17 @@
         <f aca="false">'Tháng 8'!$D$5</f>
         <v>0</v>
       </c>
+      <c r="J11" s="43" t="n">
+        <f aca="false">'Tháng 8'!$D$6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="39" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B12" s="39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C12" s="40" t="n">
         <v>46195</v>
@@ -55214,7 +55336,7 @@
         <v>0</v>
       </c>
       <c r="F12" s="42" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="G12" s="43" t="n">
         <f aca="false">'Tháng 9'!$D$3</f>
@@ -55228,13 +55350,17 @@
         <f aca="false">'Tháng 9'!$D$5</f>
         <v>0</v>
       </c>
+      <c r="J12" s="43" t="n">
+        <f aca="false">'Tháng 9'!$D$6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="42" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B13" s="42" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C13" s="17" t="n">
         <v>46204</v>
@@ -55247,7 +55373,7 @@
         <v>0</v>
       </c>
       <c r="F13" s="42" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="G13" s="43" t="n">
         <f aca="false">'Tháng 10'!$D$3</f>
@@ -55261,13 +55387,17 @@
         <f aca="false">'Tháng 10'!$D$5</f>
         <v>0</v>
       </c>
+      <c r="J13" s="43" t="n">
+        <f aca="false">'Tháng 10'!$D$6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="42" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B14" s="42" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C14" s="17" t="n">
         <v>46211</v>
@@ -55280,7 +55410,7 @@
         <v>0</v>
       </c>
       <c r="F14" s="42" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="G14" s="43" t="n">
         <f aca="false">'Tháng 11'!$D$3</f>
@@ -55294,13 +55424,17 @@
         <f aca="false">'Tháng 11'!$D$5</f>
         <v>0</v>
       </c>
+      <c r="J14" s="43" t="n">
+        <f aca="false">'Tháng 11'!$D$6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="42" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B15" s="42" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C15" s="17" t="n">
         <v>46218</v>
@@ -55313,7 +55447,7 @@
         <v>97000000</v>
       </c>
       <c r="F15" s="42" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="G15" s="43" t="n">
         <f aca="false">'Tháng 12'!$D$3</f>
@@ -55327,13 +55461,17 @@
         <f aca="false">'Tháng 12'!$D$5</f>
         <v>0</v>
       </c>
+      <c r="J15" s="43" t="n">
+        <f aca="false">'Tháng 12'!$D$6</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="42" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B16" s="42" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C16" s="17" t="n">
         <v>46225</v>
@@ -55348,10 +55486,10 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="39" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B17" s="39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C17" s="40" t="n">
         <v>46235</v>
@@ -55364,18 +55502,19 @@
         <v>0</v>
       </c>
       <c r="F17" s="35" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="G17" s="35"/>
       <c r="H17" s="35"/>
       <c r="I17" s="35"/>
+      <c r="J17" s="35"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="39" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B18" s="39" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C18" s="40" t="n">
         <v>46242</v>
@@ -55388,7 +55527,7 @@
         <v>0</v>
       </c>
       <c r="F18" s="31" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="G18" s="32" t="n">
         <f aca="false">SUM($G$9:$G$9)</f>
@@ -55400,15 +55539,19 @@
       </c>
       <c r="I18" s="32" t="n">
         <f aca="false">SUM($I$9:$I$9)</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="32" t="n">
+        <f aca="false">SUM($J$9:$J$9)</f>
         <v>6000000</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="39" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B19" s="39" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C19" s="40" t="n">
         <v>46249</v>
@@ -55421,7 +55564,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="31" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="G19" s="32" t="n">
         <f aca="false">SUM($G$10:$G$12)</f>
@@ -55433,15 +55576,19 @@
       </c>
       <c r="I19" s="32" t="n">
         <f aca="false">SUM($I$10:$I$12)</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="32" t="n">
+        <f aca="false">SUM($J$10:$J$12)</f>
         <v>47000000</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="39" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="B20" s="39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C20" s="40" t="n">
         <v>46256</v>
@@ -55454,7 +55601,7 @@
         <v>0</v>
       </c>
       <c r="F20" s="31" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="G20" s="32" t="n">
         <f aca="false">SUM($G$13:$G$15)</f>
@@ -55468,13 +55615,17 @@
         <f aca="false">SUM($I$13:$I$15)</f>
         <v>0</v>
       </c>
+      <c r="J20" s="32" t="n">
+        <f aca="false">SUM($J$13:$J$15)</f>
+        <v>0</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="42" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B21" s="42" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C21" s="17" t="n">
         <v>46266</v>
@@ -55489,10 +55640,10 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="42" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B22" s="42" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C22" s="17" t="n">
         <v>46273</v>
@@ -55505,18 +55656,19 @@
         <v>0</v>
       </c>
       <c r="F22" s="35" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="G22" s="35"/>
       <c r="H22" s="35"/>
       <c r="I22" s="35"/>
+      <c r="J22" s="35"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="42" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B23" s="42" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C23" s="17" t="n">
         <v>46280</v>
@@ -55529,7 +55681,7 @@
         <v>0</v>
       </c>
       <c r="F23" s="44" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="G23" s="45" t="n">
         <f aca="false">SUM($G$18:$G$20)</f>
@@ -55541,15 +55693,19 @@
       </c>
       <c r="I23" s="45" t="n">
         <f aca="false">SUM($I$18:$I$20)</f>
+        <v>0</v>
+      </c>
+      <c r="J23" s="45" t="n">
+        <f aca="false">SUM($J$18:$J$20)</f>
         <v>53000000</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="42" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B24" s="42" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C24" s="17" t="n">
         <v>46287</v>
@@ -55564,10 +55720,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="39" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B25" s="39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C25" s="40" t="n">
         <v>46296</v>
@@ -55580,15 +55736,15 @@
         <v>0</v>
       </c>
       <c r="F25" s="46" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="39" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B26" s="39" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C26" s="40" t="n">
         <v>46303</v>
@@ -55603,10 +55759,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="39" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B27" s="39" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C27" s="40" t="n">
         <v>46310</v>
@@ -55621,10 +55777,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="39" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B28" s="39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C28" s="40" t="n">
         <v>46317</v>
@@ -55639,10 +55795,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="42" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B29" s="42" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C29" s="17" t="n">
         <v>46327</v>
@@ -55657,10 +55813,10 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="42" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B30" s="42" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C30" s="17" t="n">
         <v>46334</v>
@@ -55675,10 +55831,10 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="42" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B31" s="42" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C31" s="17" t="n">
         <v>46341</v>
@@ -55693,10 +55849,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="42" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="B32" s="42" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C32" s="17" t="n">
         <v>46348</v>
@@ -55711,10 +55867,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B33" s="39" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="C33" s="40" t="n">
         <v>46357</v>
@@ -55729,10 +55885,10 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B34" s="39" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C34" s="40" t="n">
         <v>46364</v>
@@ -55747,10 +55903,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B35" s="39" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="C35" s="40" t="n">
         <v>46371</v>
@@ -55765,10 +55921,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="39" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B36" s="39" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C36" s="40" t="n">
         <v>46378</v>
@@ -55788,9 +55944,9 @@
     <mergeCell ref="A4:B4"/>
     <mergeCell ref="A5:B5"/>
     <mergeCell ref="A7:E7"/>
-    <mergeCell ref="F7:I7"/>
-    <mergeCell ref="F17:I17"/>
-    <mergeCell ref="F22:I22"/>
+    <mergeCell ref="F7:J7"/>
+    <mergeCell ref="F17:J17"/>
+    <mergeCell ref="F22:J22"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>